<commit_message>
updated the RTM workbook with the tests
updated the RTM workbook with the tests that succeded so far. Record first M3 test execution in RTM v3.0. Unit cases UT-01, UT-03 and UT-04 passed locally (20 passed, 1 skipped); IT-02 is recorded as blocked until a test database is configured.
</commit_message>
<xml_diff>
--- a/Docs/Risks/RTM/CivicConnect-RTM-v3.0.xlsx
+++ b/Docs/Risks/RTM/CivicConnect-RTM-v3.0.xlsx
@@ -1093,7 +1093,7 @@
       </c>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>UT-04 RequestAccessTests: pending first run on frontend-milestone-3-development. BB-05, E2E-01: not run (B1)</t>
+          <t>UT-04 RequestAccessTests: 8/8 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). BB-05, E2E-01: not run (B1)</t>
         </is>
       </c>
       <c r="V6" s="5" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>UT-04 RequestAccessTests: pending first run on frontend-milestone-3-development. BB-03: not run (needs a running RC, B2)</t>
+          <t>UT-04 RequestAccessTests: 8/8 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). BB-03: not run (needs a running RC, B2)</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
@@ -1877,7 +1877,7 @@
       </c>
       <c r="U13" s="5" t="inlineStr">
         <is>
-          <t>UT-03 AssignmentServiceTests: pending run. IT-02 ConcurrentAcceptTests: skipped in CI (no test DB, B3), counts as Blocked</t>
+          <t>UT-03 AssignmentServiceTests: 4/4 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). IT-02 ConcurrentAcceptTests: skipped (CIVICCONNECT_TEST_DB not set), counts as Blocked (B3)</t>
         </is>
       </c>
       <c r="V13" s="5" t="inlineStr">
@@ -1989,7 +1989,7 @@
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>UT-01 StatusTransitionTests: pending run. BB-04, E2E-02: not run (not wired)</t>
+          <t>UT-01 StatusTransitionTests: 8/8 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). BB-04, E2E-02: not run (not wired)</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
@@ -2213,7 +2213,7 @@
       </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>UT-04 RequestAccessTests: pending first run on frontend-milestone-3-development. IT-03: not run (no endpoint)</t>
+          <t>UT-04 RequestAccessTests: 8/8 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). IT-03: not run (no endpoint)</t>
         </is>
       </c>
       <c r="V16" s="5" t="inlineStr">
@@ -3557,7 +3557,7 @@
       </c>
       <c r="U28" s="5" t="inlineStr">
         <is>
-          <t>UT-04 RequestAccessTests: pending first run on frontend-milestone-3-development. BB-05: not run (B1)</t>
+          <t>UT-04 RequestAccessTests: 8/8 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). BB-05: not run (B1)</t>
         </is>
       </c>
       <c r="V28" s="5" t="inlineStr">
@@ -3781,7 +3781,7 @@
       </c>
       <c r="U30" s="5" t="inlineStr">
         <is>
-          <t>UT-03: pending run. IT-02: skipped in CI (B3), counts as Blocked</t>
+          <t>UT-03 AssignmentServiceTests: 4/4 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). IT-02 ConcurrentAcceptTests: skipped (CIVICCONNECT_TEST_DB not set), counts as Blocked (B3)</t>
         </is>
       </c>
       <c r="V30" s="5" t="inlineStr">
@@ -3893,7 +3893,7 @@
       </c>
       <c r="U31" s="5" t="inlineStr">
         <is>
-          <t>UT-04 RequestAccessTests: pending first run on frontend-milestone-3-development. IT-03: not run (no endpoint)</t>
+          <t>UT-04 RequestAccessTests: 8/8 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). IT-03: not run (no endpoint)</t>
         </is>
       </c>
       <c r="V31" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Give ConcurrentAcceptTests staff a category scope
Give ConcurrentAcceptTests staff a category scope and record IT-02. Since FR-008 scoping, unscoped staff are refused, so each competitor is now scoped to the test category; IT-02 passes against local PostgreSQL (21/21) and the RTM records it.
</commit_message>
<xml_diff>
--- a/Docs/Risks/RTM/CivicConnect-RTM-v3.0.xlsx
+++ b/Docs/Risks/RTM/CivicConnect-RTM-v3.0.xlsx
@@ -1877,12 +1877,12 @@
       </c>
       <c r="U13" s="5" t="inlineStr">
         <is>
-          <t>UT-03 AssignmentServiceTests: 4/4 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). IT-02 ConcurrentAcceptTests: skipped (CIVICCONNECT_TEST_DB not set), counts as Blocked (B3)</t>
+          <t>UT-03 AssignmentServiceTests: 4/4 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). IT-02 ConcurrentAcceptTests: passed against local PostgreSQL 17 (dotnet test, 2026-10-12, eeb9362 plus the ConcurrentAcceptTests scope fix; 21 total: 21 passed, 0 skipped). Still skipped in CI until CI has a test database (B3)</t>
         </is>
       </c>
       <c r="V13" s="5" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>IN: IT-02 passes locally, not yet in CI (B3)</t>
         </is>
       </c>
     </row>
@@ -3781,12 +3781,12 @@
       </c>
       <c r="U30" s="5" t="inlineStr">
         <is>
-          <t>UT-03 AssignmentServiceTests: 4/4 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). IT-02 ConcurrentAcceptTests: skipped (CIVICCONNECT_TEST_DB not set), counts as Blocked (B3)</t>
+          <t>UT-03 AssignmentServiceTests: 4/4 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). IT-02 ConcurrentAcceptTests: passed against local PostgreSQL 17 (dotnet test, 2026-10-12, eeb9362 plus the ConcurrentAcceptTests scope fix; 21 total: 21 passed, 0 skipped). Still skipped in CI until CI has a test database (B3)</t>
         </is>
       </c>
       <c r="V30" s="5" t="inlineStr">
         <is>
-          <t>IN: IT-02 blocked (B3)</t>
+          <t>IN: IT-02 passes locally, not yet in CI (B3)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Added a development user switcher and record the M3 acceptance checks.
Add a development user switcher and record the M3 acceptance checks. BB-03, AC-011.1 and AC-011.2 pass against the local build; AC-010.1 is partial because the details page omits the requester and category (DEF-001)
</commit_message>
<xml_diff>
--- a/Docs/Risks/RTM/CivicConnect-RTM-v3.0.xlsx
+++ b/Docs/Risks/RTM/CivicConnect-RTM-v3.0.xlsx
@@ -1541,7 +1541,7 @@
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>UT-04 RequestAccessTests: 8/8 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). BB-03: not run (needs a running RC, B2)</t>
+          <t>UT-04 RequestAccessTests: 8/8 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). BB-03a to BB-03e: Pass (Test/Evidence/M3_Acceptance_Checks.md, local Development build, 2026-10-12)</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
@@ -1755,7 +1755,7 @@
       </c>
       <c r="S12" s="5" t="inlineStr">
         <is>
-          <t>E2E-02 (walk-through)</t>
+          <t>AC-010.1 check, E2E-02 (walk-through)</t>
         </is>
       </c>
       <c r="T12" s="5" t="inlineStr">
@@ -1765,12 +1765,12 @@
       </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>Not run: needs a running RC (B2)</t>
+          <t>AC-010.1: Partial, requester and category not shown (Test/Evidence/M3_Acceptance_Checks.md, local Development build, 2026-10-12)</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>IN</t>
+          <t>IN: AC-010.1 partial, DEF-001 (proposed, Minor)</t>
         </is>
       </c>
     </row>
@@ -1877,7 +1877,7 @@
       </c>
       <c r="U13" s="5" t="inlineStr">
         <is>
-          <t>UT-03 AssignmentServiceTests: 4/4 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). IT-02 ConcurrentAcceptTests: passed against local PostgreSQL 17 (dotnet test, 2026-10-12, eeb9362 plus the ConcurrentAcceptTests scope fix; 21 total: 21 passed, 0 skipped). Still skipped in CI until CI has a test database (B3)</t>
+          <t>UT-03 AssignmentServiceTests: 4/4 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). IT-02 ConcurrentAcceptTests: passed against local PostgreSQL 17 (dotnet test, 2026-10-12, eeb9362 plus the ConcurrentAcceptTests scope fix; 21 total: 21 passed, 0 skipped). Still skipped in CI until CI has a test database (B3). AC-011.1 and AC-011.2 (UI): Pass (Test/Evidence/M3_Acceptance_Checks.md, local Development build, 2026-10-12)</t>
         </is>
       </c>
       <c r="V13" s="5" t="inlineStr">
@@ -3893,7 +3893,7 @@
       </c>
       <c r="U31" s="5" t="inlineStr">
         <is>
-          <t>UT-04 RequestAccessTests: 8/8 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). IT-03: not run (no endpoint)</t>
+          <t>UT-04 RequestAccessTests: 8/8 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). IT-03: not run (no endpoint). Out-of-scope accept refused, request unchanged: Pass (Test/Evidence/M3_Acceptance_Checks.md, local Development build, 2026-10-12)</t>
         </is>
       </c>
       <c r="V31" s="5" t="inlineStr">

</xml_diff>

<commit_message>
updated the change register, rtm and added conformance
Settle CR-001 to CR-011 and add the M3 baseline conformance table. Change Register v3.0 records each decision with evidence and raises CR-012 (closing rule), CR-013 (deferred Musts) and CR-014 (single deployable); the RTM statuses now point to them.
</commit_message>
<xml_diff>
--- a/Docs/Risks/RTM/CivicConnect-RTM-v3.0.xlsx
+++ b/Docs/Risks/RTM/CivicConnect-RTM-v3.0.xlsx
@@ -1658,7 +1658,7 @@
       </c>
       <c r="V11" s="5" t="inlineStr">
         <is>
-          <t>OUT: not in M3 scope (Scope Freeze v1.0)</t>
+          <t>OUT: deferred to M4 by CR-013 (proposed), Scope Freeze v1.0</t>
         </is>
       </c>
     </row>
@@ -2106,7 +2106,7 @@
       </c>
       <c r="V15" s="5" t="inlineStr">
         <is>
-          <t>OUT: not in M3 scope (Scope Freeze v1.0)</t>
+          <t>OUT: deferred to M4 by CR-013 (proposed), Scope Freeze v1.0</t>
         </is>
       </c>
     </row>
@@ -2218,7 +2218,7 @@
       </c>
       <c r="V16" s="5" t="inlineStr">
         <is>
-          <t>IN*: gap, comes with FR-012 wiring</t>
+          <t>IN*: gap, comes with FR-012 wiring; AC-014.2 reworded by CR-012 (proposed)</t>
         </is>
       </c>
     </row>
@@ -2330,7 +2330,7 @@
       </c>
       <c r="V17" s="5" t="inlineStr">
         <is>
-          <t>OUT: not in M3 scope (Scope Freeze v1.0)</t>
+          <t>OUT: deferred to M4 by CR-013 (proposed), Scope Freeze v1.0</t>
         </is>
       </c>
     </row>
@@ -2442,7 +2442,7 @@
       </c>
       <c r="V18" s="5" t="inlineStr">
         <is>
-          <t>OUT: not in M3 scope (Scope Freeze v1.0)</t>
+          <t>OUT: deferred to M4 by CR-013 (proposed), Scope Freeze v1.0</t>
         </is>
       </c>
     </row>
@@ -2554,7 +2554,7 @@
       </c>
       <c r="V19" s="5" t="inlineStr">
         <is>
-          <t>OUT: not in M3 scope (Scope Freeze v1.0)</t>
+          <t>OUT: deferred to M4 by CR-013 (proposed), Scope Freeze v1.0</t>
         </is>
       </c>
     </row>
@@ -2778,7 +2778,7 @@
       </c>
       <c r="V21" s="5" t="inlineStr">
         <is>
-          <t>OUT: not in M3 scope (Scope Freeze v1.0)</t>
+          <t>OUT: deferred to M4 by CR-013 (proposed), Scope Freeze v1.0</t>
         </is>
       </c>
     </row>
@@ -2890,7 +2890,7 @@
       </c>
       <c r="V22" s="5" t="inlineStr">
         <is>
-          <t>OUT: Scope Freeze v1.0</t>
+          <t>OUT: deferred to M4 by CR-013 (proposed), Scope Freeze v1.0</t>
         </is>
       </c>
     </row>
@@ -3002,7 +3002,7 @@
       </c>
       <c r="V23" s="5" t="inlineStr">
         <is>
-          <t>OUT: not in M3 scope (Scope Freeze v1.0)</t>
+          <t>OUT: deferred to M4 by CR-013 (proposed), Scope Freeze v1.0</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Record the release candidate evidence.
All 26 acceptance checks and PT-01 pass on the merged build; the RTM now cites them and marks FR-007, FR-009 and FR-013 as built.
</commit_message>
<xml_diff>
--- a/Docs/Risks/RTM/CivicConnect-RTM-v3.0.xlsx
+++ b/Docs/Risks/RTM/CivicConnect-RTM-v3.0.xlsx
@@ -522,7 +522,7 @@
     <row r="1" ht="17.25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CivicConnect Requirements Traceability Matrix (RTM) - M3 release candidate (live) - v3.0</t>
+          <t>CivicConnect Requirements Traceability Matrix (RTM) - M3 release candidate (live) - v3.0. Evidence: 76/76 automated tests pass locally on the release candidate; integration and E2E tests skip in CI until it has a test database (B3). Acceptance: Test/Evidence/M3_Acceptance_Checks.md</t>
         </is>
       </c>
     </row>
@@ -742,7 +742,7 @@
       </c>
       <c r="R3" s="5" t="inlineStr">
         <is>
-          <t>SubmissionService.SubmitAsync; Pages/Requests/Submit; POST /api/v1/requests; Request.Location and request_reference_seq (migration AddRequestLocation)</t>
+          <t>SubmissionService; Pages/Requests/Submit; POST /api/v1/requests; Location and reference sequence (migration AddStaffScopesLocationAndReferences)</t>
         </is>
       </c>
       <c r="S3" s="5" t="inlineStr">
@@ -757,7 +757,7 @@
       </c>
       <c r="U3" s="5" t="inlineStr">
         <is>
-          <t>UT-05 1/1, BB-01 5/5 and BB-02 4/4 passed in SubmissionServiceTests (local dotnet test, 2026-10-12, Release, 593e739 plus the requester port; 42 passed, 0 skipped). AC-001.1, AC-001.2, BB-02 (page) and IT-01 (manual API): Pass (Test/Evidence/M3_Acceptance_Checks.md round 2, 2026-10-12). IT-01 automated and E2E-01: not run</t>
+          <t>UT-05, BB-01, BB-02, IT-01, E2E-01 pass (automated). AC-001.1, AC-001.2, BB-02 pass (acceptance)</t>
         </is>
       </c>
       <c r="V3" s="5" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="U4" s="5" t="inlineStr">
         <is>
-          <t>UT-02 1/1 passed (local dotnet test, 2026-10-12, Release, 593e739 plus the requester port; 42 passed, 0 skipped). AC-002.1 and AC-002.2: Pass (Test/Evidence/M3_Acceptance_Checks.md round 2, 2026-10-12)</t>
+          <t>UT-02 pass (automated). AC-002.1, AC-002.2 pass (acceptance)</t>
         </is>
       </c>
       <c r="V4" s="5" t="inlineStr">
@@ -981,7 +981,7 @@
       </c>
       <c r="U5" s="5" t="inlineStr">
         <is>
-          <t>AC-003.1 and AC-003.2: Pass (Test/Evidence/M3_Acceptance_Checks.md round 2, 2026-10-12). E2E-01: not run</t>
+          <t>E2E-01 pass (automated). AC-003.1, AC-003.2 pass (acceptance)</t>
         </is>
       </c>
       <c r="V5" s="5" t="inlineStr">
@@ -1093,12 +1093,12 @@
       </c>
       <c r="U6" s="5" t="inlineStr">
         <is>
-          <t>UT-04 RequestAccessTests 12/12 passed (local dotnet test, 2026-10-12, Release, 593e739 plus the requester port; 42 passed, 0 skipped). AC-004.1: Pass (Test/Evidence/M3_Acceptance_Checks.md round 2, 2026-10-12). BB-05: not run (the seed has one requester). E2E-01: not run</t>
+          <t>BB-05, E2E-01 pass (automated). AC-004.1, BB-05 pass (acceptance)</t>
         </is>
       </c>
       <c r="V6" s="5" t="inlineStr">
         <is>
-          <t>IN: BB-05 needs a second seeded requester</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -1414,7 +1414,7 @@
       </c>
       <c r="R9" s="5" t="inlineStr">
         <is>
-          <t>Not in app/</t>
+          <t>Assignment and status changes write RequesterFeedback; Pages/Requests/Details lists the updates</t>
         </is>
       </c>
       <c r="S9" s="5" t="inlineStr">
@@ -1424,17 +1424,17 @@
       </c>
       <c r="T9" s="5" t="inlineStr">
         <is>
-          <t>A feedback item with a timestamp appears for the requester after a status change</t>
+          <t>A timestamped update for each change, shown on the requester's next visit</t>
         </is>
       </c>
       <c r="U9" s="5" t="inlineStr">
         <is>
-          <t>Not run: blocked by B1 and FR-012 wiring</t>
+          <t>E2E-02 pass (automated). AC-007.1 pass (acceptance). AC-007.2 not built (CR-009)</t>
         </is>
       </c>
       <c r="V9" s="5" t="inlineStr">
         <is>
-          <t>IN* (stretch): blocked (B1)</t>
+          <t>IN: AC-007.2 deferred (CR-009)</t>
         </is>
       </c>
     </row>
@@ -1526,12 +1526,12 @@
       </c>
       <c r="R10" s="5" t="inlineStr">
         <is>
-          <t>Pages/Staff/Queue.cshtml.cs scoped query; Domain/Access/StaffCategoryScope; AuthorisationPolicy with RequestAccess.MayView; Staff/Details returns 404 outside scope</t>
+          <t>IQueueRepository and Staff/Queue scoped by category; scope check in AuthorisationPolicy; Staff/Details 404 outside scope</t>
         </is>
       </c>
       <c r="S10" s="5" t="inlineStr">
         <is>
-          <t>UT-04, BB-03</t>
+          <t>UT-04, BB-03, QueueTests</t>
         </is>
       </c>
       <c r="T10" s="5" t="inlineStr">
@@ -1541,12 +1541,12 @@
       </c>
       <c r="U10" s="5" t="inlineStr">
         <is>
-          <t>UT-04 RequestAccessTests: 8/8 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). BB-03a to BB-03e: Pass (Test/Evidence/M3_Acceptance_Checks.md, local Development build, 2026-10-12)</t>
+          <t>UT-04, QueueTests pass (automated). BB-03a to BB-03e pass (acceptance)</t>
         </is>
       </c>
       <c r="V10" s="5" t="inlineStr">
         <is>
-          <t>IN: B4 closed by category scope</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -1638,27 +1638,27 @@
       </c>
       <c r="R11" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>IQueueRepository.SearchAsync (filter, search, sort, paging); GET /api/v1/queue; Staff/Queue filter bar</t>
         </is>
       </c>
       <c r="S11" s="5" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>QueueTests, ApiTests, StaffScreensTests</t>
         </is>
       </c>
       <c r="T11" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Only matching requests in the staff member's scope, in the chosen order; a message when none match</t>
         </is>
       </c>
       <c r="U11" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>QueueTests, ApiTests, StaffScreensTests pass (automated). Search and filter pass (acceptance)</t>
         </is>
       </c>
       <c r="V11" s="5" t="inlineStr">
         <is>
-          <t>OUT: deferred to M4 by CR-013 (proposed), Scope Freeze v1.0</t>
+          <t>IN: built after the freeze; remove from CR-013</t>
         </is>
       </c>
     </row>
@@ -1765,12 +1765,12 @@
       </c>
       <c r="U12" s="5" t="inlineStr">
         <is>
-          <t>AC-010.1: Partial in round 1 (DEF-001); retest Pass after the fix (Test/Evidence/M3_Acceptance_Checks.md round 2, 2026-10-12)</t>
+          <t>AC-010.1 pass (acceptance); DEF-001 fixed</t>
         </is>
       </c>
       <c r="V12" s="5" t="inlineStr">
         <is>
-          <t>IN: DEF-001 fixed</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -1877,12 +1877,12 @@
       </c>
       <c r="U13" s="5" t="inlineStr">
         <is>
-          <t>UT-03 AssignmentServiceTests: 4/4 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). IT-02 ConcurrentAcceptTests: passed against local PostgreSQL 17 (dotnet test, 2026-10-12, eeb9362 plus the ConcurrentAcceptTests scope fix; 21 total: 21 passed, 0 skipped). Still skipped in CI until CI has a test database (B3). AC-011.1 and AC-011.2 (UI): Pass (Test/Evidence/M3_Acceptance_Checks.md, local Development build, 2026-10-12)</t>
+          <t>UT-03, IT-02, eight-staff API race pass (automated). AC-011.1, AC-011.2 pass (acceptance)</t>
         </is>
       </c>
       <c r="V13" s="5" t="inlineStr">
         <is>
-          <t>IN: IT-02 passes locally, not yet in CI (B3)</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -1974,7 +1974,7 @@
       </c>
       <c r="R14" s="5" t="inlineStr">
         <is>
-          <t>StatusTransitionService.MoveAsync wired to Pages/Staff/Details (next-status form) and PATCH /api/v1/requests/{id}/status</t>
+          <t>StatusTransitionService.MoveAsync; Staff/Details status form; POST /api/v1/requests/{id}/status</t>
         </is>
       </c>
       <c r="S14" s="5" t="inlineStr">
@@ -1989,7 +1989,7 @@
       </c>
       <c r="U14" s="5" t="inlineStr">
         <is>
-          <t>UT-01 StatusTransitionTests 8/8 and StatusTransitionServiceTests 2/2 passed (local dotnet test, 2026-10-12, Release, 593e739 plus the requester port; 42 passed, 0 skipped). AC-012.1 and AC-012.2 (BB-04 flow): Pass (Test/Evidence/M3_Acceptance_Checks.md round 2, 2026-10-12). E2E-02: not run</t>
+          <t>UT-01, StatusTransitionServiceTests, LifecycleTests, E2E-02 pass (automated). AC-012.1, AC-012.2 pass (acceptance)</t>
         </is>
       </c>
       <c r="V14" s="5" t="inlineStr">
@@ -2086,27 +2086,27 @@
       </c>
       <c r="R15" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>NoteService; POST /api/v1/requests/{id}/notes; Staff/Details add-note form</t>
         </is>
       </c>
       <c r="S15" s="5" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>NoteServiceTests, ApiTests, StaffScreensTests</t>
         </is>
       </c>
       <c r="T15" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>A note is saved to the history with author and time and is never edited</t>
         </is>
       </c>
       <c r="U15" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>NoteServiceTests, ApiTests, StaffScreensTests pass (automated). Add a note pass (acceptance)</t>
         </is>
       </c>
       <c r="V15" s="5" t="inlineStr">
         <is>
-          <t>OUT: deferred to M4 by CR-013 (proposed), Scope Freeze v1.0</t>
+          <t>IN: built after the freeze; remove from CR-013</t>
         </is>
       </c>
     </row>
@@ -2198,7 +2198,7 @@
       </c>
       <c r="R16" s="5" t="inlineStr">
         <is>
-          <t>Close checked as its own action (RequestAction.Close, RequestAccess.MayWorkOn); resolution note stored on the history entry</t>
+          <t>Close checked as its own action: the owner in scope or an administrator (CR-012); resolving needs a note</t>
         </is>
       </c>
       <c r="S16" s="5" t="inlineStr">
@@ -2213,12 +2213,12 @@
       </c>
       <c r="U16" s="5" t="inlineStr">
         <is>
-          <t>UT-04 StatusTransitionServiceTests 2/2 and RequestAccessTests 12/12 passed (local dotnet test, 2026-10-12, Release, 593e739 plus the requester port; 42 passed, 0 skipped). AC-014.2 and IT-03 (manual API, 403): Pass. AC-014.1: Partial, no requester feedback because FR-007 is not built (Test/Evidence/M3_Acceptance_Checks.md round 2, 2026-10-12)</t>
+          <t>IT-03, E2E-02, AuthorisationTests pass (automated). AC-014.1, AC-014.2, administrator close pass (acceptance)</t>
         </is>
       </c>
       <c r="V16" s="5" t="inlineStr">
         <is>
-          <t>IN: AC-014.1 partial (FR-007); AC-014.2 reworded by CR-012 (proposed)</t>
+          <t>IN: AC-014.2 reworded by CR-012 (proposed)</t>
         </is>
       </c>
     </row>
@@ -3557,12 +3557,12 @@
       </c>
       <c r="U28" s="5" t="inlineStr">
         <is>
-          <t>UT-04 RequestAccessTests 12/12 passed (local dotnet test, 2026-10-12, Release, 593e739 plus the requester port; 42 passed, 0 skipped). BB-05: not run (the seed has one requester)</t>
+          <t>UT-04, BB-05 pass (automated). BB-05 pass (acceptance)</t>
         </is>
       </c>
       <c r="V28" s="5" t="inlineStr">
         <is>
-          <t>IN: BB-05 needs a second seeded requester</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -3654,12 +3654,12 @@
       </c>
       <c r="R29" s="5" t="inlineStr">
         <is>
-          <t>Staff queue query (indexed, capped at 50 rows)</t>
+          <t>IQueueRepository query, indexed and paged at 20 rows</t>
         </is>
       </c>
       <c r="S29" s="5" t="inlineStr">
         <is>
-          <t>PT-01</t>
+          <t>PT-01, QueueTests</t>
         </is>
       </c>
       <c r="T29" s="5" t="inlineStr">
@@ -3669,12 +3669,12 @@
       </c>
       <c r="U29" s="5" t="inlineStr">
         <is>
-          <t>Not run: no staging RC (B2)</t>
+          <t>PT-01 pass: p95 0.064 s with 5 users, 0 errors (Test/Evidence/PT-01_Results.md). QueueTests 1,000-request check pass</t>
         </is>
       </c>
       <c r="V29" s="5" t="inlineStr">
         <is>
-          <t>IN*: blocked (B2)</t>
+          <t>IN: measured locally; staging pending (B2)</t>
         </is>
       </c>
     </row>
@@ -3781,12 +3781,12 @@
       </c>
       <c r="U30" s="5" t="inlineStr">
         <is>
-          <t>UT-03 AssignmentServiceTests: 4/4 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). IT-02 ConcurrentAcceptTests: passed against local PostgreSQL 17 (dotnet test, 2026-10-12, eeb9362 plus the ConcurrentAcceptTests scope fix; 21 total: 21 passed, 0 skipped). Still skipped in CI until CI has a test database (B3)</t>
+          <t>UT-03, IT-02, eight-staff API race pass (automated)</t>
         </is>
       </c>
       <c r="V30" s="5" t="inlineStr">
         <is>
-          <t>IN: IT-02 passes locally, not yet in CI (B3)</t>
+          <t>IN</t>
         </is>
       </c>
     </row>
@@ -3893,7 +3893,7 @@
       </c>
       <c r="U31" s="5" t="inlineStr">
         <is>
-          <t>UT-04 RequestAccessTests: 8/8 passed (local dotnet test, 2026-10-12, commit 0339355, .NET 10.0.12 (21 total: 20 passed, 0 failed, 1 skipped)). IT-03 (manual): 403 for Staff Two and the requester (Test/Evidence/M3_Acceptance_Checks.md round 2, 2026-10-12). Out-of-scope accept refused, request unchanged: Pass (Test/Evidence/M3_Acceptance_Checks.md, local Development build, 2026-10-12)</t>
+          <t>UT-04, IT-03, AuthorisationTests pass (automated). Out-of-scope accept refused, AC-014.2 pass (acceptance)</t>
         </is>
       </c>
       <c r="V31" s="5" t="inlineStr">

</xml_diff>